<commit_message>
New HubSpot Updated Selectors
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\botuser_5\Documents\UiPath\FIN_Invoicing_ContractSent_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64418B2B-53AB-4C76-A036-C1B961ACB5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8543AFEC-77BC-4B84-9512-05CB71870FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="131">
   <si>
     <t>Name</t>
   </si>
@@ -429,6 +429,21 @@
   </si>
   <si>
     <t>InvoicesReportFilename</t>
+  </si>
+  <si>
+    <t>ExcelFileExtension</t>
+  </si>
+  <si>
+    <t>xlsx</t>
+  </si>
+  <si>
+    <t>OutputFolderPath</t>
+  </si>
+  <si>
+    <t>Data\Output\</t>
+  </si>
+  <si>
+    <t>Output Folder Path</t>
   </si>
 </sst>
 </file>
@@ -446,6 +461,7 @@
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="6"/>
@@ -1901,7 +1917,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z991"/>
+  <dimension ref="A1:Z993"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -2214,61 +2230,81 @@
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B30" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="C30" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B31" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C31" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C32" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B33" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="C33" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1">
       <c r="A34" t="s">
+        <v>109</v>
+      </c>
+      <c r="B34" t="s">
+        <v>110</v>
+      </c>
+      <c r="C34" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A35" t="s">
+        <v>126</v>
+      </c>
+      <c r="B35" t="s">
+        <v>127</v>
+      </c>
+      <c r="C35" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A36" t="s">
         <v>114</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B36" t="s">
         <v>115</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C36" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="36" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="37" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="38" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="39" spans="1:3" ht="14.25" customHeight="1"/>
@@ -3224,6 +3260,8 @@
     <row r="989" ht="14.25" customHeight="1"/>
     <row r="990" ht="14.25" customHeight="1"/>
     <row r="991" ht="14.25" customHeight="1"/>
+    <row r="992" ht="14.25" customHeight="1"/>
+    <row r="993" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>